<commit_message>
feat: ship AI advisory foundation and hardening
- add the feature-flagged transaction-case AI advisory module, route, storage, and dashboard card
- harden production env validation and CI coverage for infrastructure safeguards
- document audit prep, AI rollout, and the detailed real LLM integration plan

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/plans/TREASURYOS_JIRA_PRODUCT_OPS_WORKBOOK.xlsx
+++ b/docs/plans/TREASURYOS_JIRA_PRODUCT_OPS_WORKBOOK.xlsx
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T1_Overview" displayName="T1_Overview" ref="A1:D20" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T1_Overview" displayName="T1_Overview" ref="A1:D21" headerRowCount="1">
   <autoFilter ref="A1:D20"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Category"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T3_Active_Tickets" displayName="T3_Active_Tickets" ref="A1:N18" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T3_Active_Tickets" displayName="T3_Active_Tickets" ref="A1:N20" headerRowCount="1">
   <autoFilter ref="A1:N18"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Initiative"/>
@@ -224,7 +224,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TJiraImport" displayName="TJiraImport" ref="A1:M30" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TJiraImport" displayName="TJiraImport" ref="A1:M32" headerRowCount="1">
   <autoFilter ref="A1:M30"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Import Pass"/>
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1053,6 +1053,28 @@
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Google supports Jira; it should not replace Jira.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Solana Phase Two</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Governance-aware proposal_pending wallet state implemented; Squads rollout prep is the next active step.</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1341,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Define advisory schemas, redaction rules, feedback capture, and auditable storage for AI outputs.</t>
+          <t>Define and harden advisory schemas, redaction rules, and auditable storage; operator feedback capture remains a follow-up.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1356,7 +1378,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Add the API gateway AI module, provider abstraction, feature flags, typed outputs, and strict no-signer boundaries.</t>
+          <t>Add the API gateway AI module, provider abstraction, feature flags, typed outputs, and no-signer boundaries for the first advisory slice.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1393,7 +1415,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Launch low-risk AI features such as case summaries and report narratives before approval assistance.</t>
+          <t>Ship transaction-case advisories first and expand to additional read-only AI surfaces only after the first slice is stable.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1655,7 +1677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2410,7 +2432,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2450,7 +2472,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Railway env updated; signer loads correctly; preview mode still works on testnet settings.</t>
+          <t>Railway env updated, signer loads correctly, readiness is green, and the testnet runtime supports the completed canary path.</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2504,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2502,7 +2524,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/SOLANA_TESTNET_DEPLOYMENT_WORKLOG.md</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2522,7 +2544,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Real testnet signature stored; explorer link verified; rollback to preview mode proven.</t>
+          <t>Real testnet signature stored, whitelist entry verified, and the canary result documented.</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2576,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2569,12 +2591,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>post-canary</t>
+          <t>testnet</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2589,12 +2611,12 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>After a successful direct-signer canary, decide whether to add Squads multisig, improved wallet pending states, and KYC compliance-registry writes.</t>
+          <t>After the successful direct-signer canary, harden governance-aware wallet states, prepare the Squads testnet rollout, and decide whether to expand into broader on-chain compliance sync.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Decision recorded with scope, risks, and next tasks.</t>
+          <t>Governance-aware pending-state behavior is implemented and the next rollout steps are documented.</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2706,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Design AI storage and redaction</t>
+          <t>Harden AI storage and redaction foundation</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2694,7 +2716,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2714,12 +2736,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>design-ai-storage-redaction</t>
+          <t>harden-ai-storage-redaction-foundation</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2729,12 +2751,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Define redaction rules, advisory schemas, storage tables, feedback capture, and auditability requirements for AI outputs before implementation begins.</t>
+          <t>Implement the first advisory schema, redaction profile, persistent ai_advisories storage, and auditability model for transaction-case summaries while leaving operator feedback capture as a later increment.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Redaction policy, data model, and audit approach documented.</t>
+          <t>The first advisory slice persists safely with a redaction profile and audit trail, and the remaining feedback work is explicit.</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2778,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Implement AI module skeleton</t>
+          <t>Implement AI module foundation</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2766,7 +2788,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2786,12 +2808,12 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>implement-ai-module-skeleton</t>
+          <t>implement-ai-module-foundation</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2801,12 +2823,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Add an API gateway AI module with provider abstraction, feature flags, typed advisory outputs, and no authority over approvals or Solana signing.</t>
+          <t>Add the API gateway AI module, deterministic provider abstraction, feature flags, typed advisory outputs, and strict no-authority boundaries for approvals or Solana signing.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>AI module exists behind feature flags and respects no-signer boundaries.</t>
+          <t>The AI module ships behind flags with typed outputs, a transaction-case advisory endpoint, and no signer or approval authority.</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2850,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Ship read-only AI advisories</t>
+          <t>Ship transaction-case AI advisories</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2838,12 +2860,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ai, transaction-cases, reports, audit</t>
+          <t>ai, transaction-cases, dashboard, audit</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2858,27 +2880,27 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>ship-ai-readonly-advisories</t>
+          <t>ship-transaction-case-ai-advisories</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Implement AI module skeleton</t>
+          <t>Implement AI module foundation</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Deliver the first low-risk AI features such as transaction-case summaries or report narratives through the dashboard and API without coupling AI to approval or chain execution paths.</t>
+          <t>Deliver the first low-risk AI feature through the API and dashboard: transaction-case summaries, recommendations, risk factors, and operator checklists without coupling AI to approval or chain execution paths.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Operators can view AI summaries; no approval path depends on AI.</t>
+          <t>Operators can view the AI advisory card on transaction-case detail pages, the feature is flag-gated, and no approval path depends on AI.</t>
         </is>
       </c>
     </row>
@@ -2947,6 +2969,150 @@
       <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Warning source understood; risk classified; remediation or documented waiver agreed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Solana Testnet Enablement</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Evaluate Solana Phase Two</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Implement governance-aware wallet states</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>solana, governance, api-gateway, dashboard</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>initiative:solana-testnet, area:solana, phase:two</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>testnet</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>phase-two-wallet-statuses</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Run testnet wallet canary</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Add proposal-pending wallet semantics across shared types, API approval flow, transaction screening, audit events, and dashboard wallet views so Squads proposals no longer look fully approved.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Squads proposal approvals land in proposal_pending, operator messaging is clear, and downstream screening remains blocked until execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Solana Testnet Enablement</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Evaluate Solana Phase Two</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Prepare Squads testnet rollout</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>solana, governance, infra</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>initiative:solana-testnet, area:solana, blocked:external-values</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>testnet</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>phase-two-governance-prep</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Implement governance-aware wallet states</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Document the remaining external setup for testnet Squads rollout: create the multisig, confirm signer set and threshold, inject env values, and run the first governed wallet execution.</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Multisig details, runtime inputs, and the governed execution checklist are ready for the next rollout step.</t>
         </is>
       </c>
     </row>
@@ -2966,7 +3132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3200,7 +3366,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -3261,7 +3427,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -3281,17 +3447,17 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>docs/plans/SOLANA_TESTNET_ENABLEMENT_PLAN.md</t>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Decide whether to add Squads multisig, improved wallet pending states, and optional KYC chain sync.</t>
+          <t>After the successful direct-signer canary, harden governance-aware wallet states, prepare the Squads testnet rollout, and decide whether to expand into broader on-chain compliance sync.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Decision recorded with next steps.</t>
+          <t>Governance-aware pending-state behavior is implemented and the next rollout steps are documented.</t>
         </is>
       </c>
     </row>
@@ -3383,7 +3549,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -3403,17 +3569,17 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>docs/plans/AI_ADVISORY_LAYER_IMPLEMENTATION_PLAN.md</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Define advisory schemas, redaction rules, feedback capture, and auditable storage.</t>
+          <t>Define and harden advisory schemas, redaction rules, and auditable storage; operator feedback capture remains a follow-up.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Redaction and storage design approved.</t>
+          <t>First advisory storage and redaction ship with auditability, and the remaining feedback layer is clearly queued.</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3610,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -3464,17 +3630,17 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>docs/plans/AI_ADVISORY_LAYER_IMPLEMENTATION_PLAN.md</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Add the API gateway AI module, provider abstraction, feature flags, typed outputs, and no-signer boundaries.</t>
+          <t>Add the API gateway AI module, provider abstraction, feature flags, typed outputs, and no-signer boundaries for the first advisory slice.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>AI module foundation exists behind flags.</t>
+          <t>AI module foundation is shipped behind flags and remains outside approval and signing paths.</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3671,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -3525,17 +3691,17 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>docs/plans/AI_ADVISORY_LAYER_IMPLEMENTATION_PLAN.md</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Launch low-risk AI features such as case summaries and report narratives.</t>
+          <t>Ship transaction-case advisories first and expand to additional read-only AI surfaces only after the first slice is stable.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Operators can view read-only AI advisories.</t>
+          <t>Operators can already view transaction-case advisories and the next read-only surfaces are queued deliberately.</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4525,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -4389,7 +4555,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Railway API uses the deployed testnet program and dedicated signer with SOLANA_SYNC_ENABLED=false, and /api/health/ready is green.</t>
+          <t>Railway env updated, signer loads correctly, readiness is green, and the runtime supports the completed canary path.</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4586,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -4440,7 +4606,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/SOLANA_TESTNET_DEPLOYMENT_WORKLOG.md</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -4450,7 +4616,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Real testnet signature stored and rollback back to preview mode proven.</t>
+          <t>Real testnet signature stored, whitelist entry verified, and the canary result documented.</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4647,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -4501,17 +4667,17 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>After a successful direct-signer canary, decide whether to add Squads multisig and broader on-chain expansion.</t>
+          <t>After the successful direct-signer canary, harden governance-aware wallet states, prepare the Squads testnet rollout, and decide whether to expand into broader on-chain compliance sync.</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Decision and follow-up plan documented.</t>
+          <t>Governance-aware pending-state behavior is implemented and the next rollout steps are documented.</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4753,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Design AI storage and redaction</t>
+          <t>Harden AI storage and redaction foundation</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -4603,7 +4769,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -4623,17 +4789,17 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Define redaction rules, advisory schemas, storage tables, feedback capture, and auditability requirements.</t>
+          <t>Implement the first advisory schema, redaction profile, persistent ai_advisories storage, and auditability model for transaction-case summaries while leaving operator feedback capture as a later increment.</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Storage and redaction design approved.</t>
+          <t>The first advisory slice persists safely with a redaction profile and audit trail, and the remaining feedback work is explicit.</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4814,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Implement AI module skeleton</t>
+          <t>Implement AI module foundation</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
@@ -4664,7 +4830,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -4684,17 +4850,17 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Add an API gateway AI module with provider abstraction, feature flags, typed advisory outputs, and no authority over approvals or Solana signing.</t>
+          <t>Add the API gateway AI module, deterministic provider abstraction, feature flags, typed advisory outputs, and strict no-authority boundaries for approvals or Solana signing.</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>AI module skeleton works behind feature flags.</t>
+          <t>The AI module ships behind flags with typed outputs, a transaction-case advisory endpoint, and no signer or approval authority.</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4875,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Ship read-only AI advisories</t>
+          <t>Ship transaction-case AI advisories</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
@@ -4725,12 +4891,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>ai, transaction-cases, reports, audit</t>
+          <t>ai, transaction-cases, dashboard, audit</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -4745,17 +4911,17 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>docs/reports/AI_ADVISORY_FOUNDATION_REPORT.md</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Deliver low-risk AI features such as transaction-case summaries or report narratives without coupling AI to approval or chain execution.</t>
+          <t>Deliver the first low-risk AI feature through the API and dashboard: transaction-case summaries, recommendations, risk factors, and operator checklists without coupling AI to approval or chain execution paths.</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Users can view read-only AI summaries in the product.</t>
+          <t>Operators can view the AI advisory card on transaction-case detail pages, the feature is flag-gated, and no approval path depends on AI.</t>
         </is>
       </c>
     </row>
@@ -4817,6 +4983,126 @@
       <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Warning source understood and risk classified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Implement governance-aware wallet states</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Evaluate Solana Phase Two</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>solana, governance, api-gateway, dashboard</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>initiative:solana-testnet, area:solana, phase:two</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>testnet</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Add proposal-pending wallet semantics across shared types, API approval flow, transaction screening, audit events, and dashboard wallet views so Squads proposals no longer look fully approved.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Squads proposal approvals land in proposal_pending, operator messaging is clear, and downstream screening remains blocked until execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Prepare Squads testnet rollout</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Evaluate Solana Phase Two</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>solana, governance, infra</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>initiative:solana-testnet, area:solana, blocked:external-values</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>testnet</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>docs/reports/PHASE_TWO_GOVERNANCE_PENDING_STATUS_REPORT.md</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Document the remaining external setup for testnet Squads rollout: create the multisig, confirm signer set and threshold, inject env values, and run the first governed wallet execution.</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Multisig details, runtime inputs, and the governed execution checklist are ready for the next rollout step.</t>
         </is>
       </c>
     </row>

</xml_diff>